<commit_message>
Tarefas foram fragmentadas em 3 , resolução de bugs envio de email
</commit_message>
<xml_diff>
--- a/Plan_RNC.xlsx
+++ b/Plan_RNC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\AUTO-RNC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1CB21F4-0D53-4944-AE38-89D2106E6902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0915D352-746C-4E15-983D-67667789C21F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="59">
   <si>
     <t>NUMERO-NF</t>
   </si>
@@ -162,15 +162,6 @@
     <t>RESPONSAVEL</t>
   </si>
   <si>
-    <t>DEVOLUÇÃO CLIENTE</t>
-  </si>
-  <si>
-    <t>69468/25</t>
-  </si>
-  <si>
-    <t>LOADER CX02X10KG</t>
-  </si>
-  <si>
     <t>KG</t>
   </si>
   <si>
@@ -195,9 +186,6 @@
     <t>Big Bag</t>
   </si>
   <si>
-    <t>DEVOLUÇÃO</t>
-  </si>
-  <si>
     <t>PASTA-ANEXOS</t>
   </si>
   <si>
@@ -222,53 +210,41 @@
     <t>RESUMO-RAPIDO</t>
   </si>
   <si>
-    <t>*DESLIGAR NUM-LOCK</t>
-  </si>
-  <si>
-    <t>Hortolândia</t>
-  </si>
-  <si>
-    <t>a01</t>
-  </si>
-  <si>
-    <t>Durante a descarga da devolução proveniente do cliente Carlos Tamotsu Kogio, realizada no veículo placa ODO0C67, foi identificada a seguinte não conformidade: A) O produto LOADER CX02X10KG (NF 594, Lote 69468/25) apresentou 3 (três) caixas rasgadas, totalizando 60kg na movimentação. No momento da inspeção, constatou-se que, apesar do dano nas embalagens secundárias (caixas), o produto interno não foi avariado. A ressalva é necessária devido à descaracterização da embalagem padrão Nitro.</t>
-  </si>
-  <si>
-    <t>03 caixas rasgadas</t>
-  </si>
-  <si>
-    <t>50kg do produto faltando</t>
-  </si>
-  <si>
-    <t>a02</t>
-  </si>
-  <si>
-    <t>ASCU0350PB</t>
-  </si>
-  <si>
-    <t>FERTICOBRE 35 A SCX25KG</t>
-  </si>
-  <si>
-    <t>VZP TRANSF HORT</t>
-  </si>
-  <si>
     <t>VZP NITRO</t>
   </si>
   <si>
-    <t>0511/25</t>
-  </si>
-  <si>
-    <t>Durante o recebimento proveniente da unidade VZP NITRO, realizado pela transportadora MMCM TRANSPORTES, veículo placa CSK4B33, foi identificada a seguinte não conformidade: A) O produto FERTICOBRE 35 A SCX25KG (NF 10605, Lote 0511/25) apresentou uma divergência no ato da descarga, totalizando a falta de 50kg (2 sacos). No momento da conferência física da carga, constatou-se a ausência dos volumes em relação ao faturamento da nota fiscal, caracterizando a falta do produto no ato da entrega.</t>
-  </si>
-  <si>
     <t>NITRO</t>
+  </si>
+  <si>
+    <t>DATA DE FRABRICAÇÃO DIVERGENTE</t>
+  </si>
+  <si>
+    <t>00104</t>
+  </si>
+  <si>
+    <t>SPEED GRAMINEA SCX25KG</t>
+  </si>
+  <si>
+    <t>74771/26</t>
+  </si>
+  <si>
+    <t>a05</t>
+  </si>
+  <si>
+    <t>Cuiabá</t>
+  </si>
+  <si>
+    <t>VZP TRANSF CBA</t>
+  </si>
+  <si>
+    <t>Durante o recebimento proveniente da unidade NITRO VZP, realizado pela transportadora MMCM, veículo placa SUF-2B15, foi identificada a seguinte não conformidade: A) O produto SPEED GRAMINEA SCX25KG (NF 10670, Lote 74771/26) apresentou divergência na informação de data de fabricação. No momento da conferência física, constatou-se que a data gravada nas sacarias é 04/03/2026, enquanto o documento fiscal (NF) indica a data de 06/03/2026. Esta inconsistência entre o físico e o faturado compromete a rastreabilidade e o padrão de conformidade Nitro.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -330,14 +306,6 @@
       <family val="1"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
@@ -351,6 +319,39 @@
       <family val="1"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <u/>
       <sz val="12"/>
       <color rgb="FFFFC000"/>
@@ -360,14 +361,15 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Segoe UI"/>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -447,7 +449,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -472,12 +474,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -489,14 +485,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -505,10 +498,30 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -516,7 +529,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -793,672 +817,633 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W19"/>
-  <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="22" width="25.77734375" style="1"/>
-    <col min="24" max="16384" width="25.77734375" style="1"/>
+    <col min="1" max="22" width="25.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="0" hidden="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.88671875" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="19" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:23" s="16" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="P1" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="R1" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="T1" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="U1" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="V1" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="17"/>
+    </row>
+    <row r="2" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="18">
+        <v>355</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="11" t="s">
+      <c r="E2" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="10">
+        <v>10670</v>
+      </c>
+      <c r="J2" s="11">
+        <v>46087</v>
+      </c>
+      <c r="K2" s="11">
+        <v>46816</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="M2" s="11">
+        <v>46085</v>
+      </c>
+      <c r="N2" s="11">
+        <v>46816</v>
+      </c>
+      <c r="O2" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="P2" s="24">
+        <v>30000</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="T2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="V2" s="12" t="str">
+        <f>IF(B2="",0,VLOOKUP(T2,Planilha1!$A$2:$B$14,2,FALSE))</f>
+        <v>PROCESSO</v>
+      </c>
+      <c r="W2"/>
+    </row>
+    <row r="3" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="12">
+        <f>IF(B3="",0,VLOOKUP(T3,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="J1" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="L1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="O1" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="S1" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="T1" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="U1" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="V1" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="W1" s="20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="21">
-        <v>349</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="12">
-        <v>989</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="12">
-        <v>594</v>
-      </c>
-      <c r="J2" s="13">
-        <v>45849</v>
-      </c>
-      <c r="K2" s="13">
-        <v>46945</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="13">
-        <v>45849</v>
-      </c>
-      <c r="N2" s="13">
-        <v>46945</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2" s="12">
-        <v>60</v>
-      </c>
-      <c r="Q2" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="R2" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="S2" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="T2" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="U2" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="V2" s="14" t="str">
-        <f>IF(B2="",0,VLOOKUP(T2,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>AVARIA</v>
-      </c>
-      <c r="W2"/>
-    </row>
-    <row r="3" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" s="21">
-        <v>350</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" s="12">
-        <v>10605</v>
-      </c>
-      <c r="J3" s="13">
-        <v>45866</v>
-      </c>
-      <c r="K3" s="13">
-        <v>46596</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="M3" s="13">
-        <v>45866</v>
-      </c>
-      <c r="N3" s="13">
-        <v>46596</v>
-      </c>
-      <c r="O3" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="P3" s="12">
-        <v>50</v>
-      </c>
-      <c r="Q3" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="S3" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="T3" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="U3" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="V3" s="14" t="str">
-        <f>IF(B3="",0,VLOOKUP(T3,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>PROCESSO</v>
-      </c>
       <c r="W3"/>
     </row>
     <row r="4" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="18"/>
-      <c r="T4" s="12"/>
-      <c r="U4" s="12"/>
-      <c r="V4" s="14">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="12">
         <f>IF(B4="",0,VLOOKUP(T4,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W4"/>
     </row>
     <row r="5" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
-      <c r="N5" s="12"/>
-      <c r="O5" s="12"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="12"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="12"/>
-      <c r="T5" s="12"/>
-      <c r="U5" s="12"/>
-      <c r="V5" s="14">
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="12">
         <f>IF(B5="",0,VLOOKUP(T5,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W5"/>
     </row>
-    <row r="6" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="12"/>
-      <c r="U6" s="12"/>
-      <c r="V6" s="14">
+    <row r="6" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="12">
         <f>IF(B6="",0,VLOOKUP(T6,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W6"/>
     </row>
-    <row r="7" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-      <c r="R7" s="12"/>
-      <c r="S7" s="12"/>
-      <c r="T7" s="12"/>
-      <c r="U7" s="12"/>
-      <c r="V7" s="14">
+    <row r="7" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="12">
         <f>IF(B7="",0,VLOOKUP(T7,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W7"/>
     </row>
-    <row r="8" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
-      <c r="U8" s="12"/>
-      <c r="V8" s="14">
+    <row r="8" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="12">
         <f>IF(B8="",0,VLOOKUP(T8,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W8"/>
     </row>
-    <row r="9" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="14">
+    <row r="9" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="12">
         <f>IF(B9="",0,VLOOKUP(T9,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W9"/>
     </row>
-    <row r="10" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="14">
+    <row r="10" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="12">
         <f>IF(B10="",0,VLOOKUP(T10,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W10"/>
     </row>
-    <row r="11" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="12"/>
-      <c r="S11" s="12"/>
-      <c r="T11" s="12"/>
-      <c r="U11" s="12"/>
-      <c r="V11" s="14">
+    <row r="11" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="12">
         <f>IF(B11="",0,VLOOKUP(T11,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W11"/>
     </row>
-    <row r="12" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
-      <c r="R12" s="12"/>
-      <c r="S12" s="12"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="12"/>
-      <c r="V12" s="14">
+    <row r="12" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="24"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="12">
         <f>IF(B12="",0,VLOOKUP(T12,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W12"/>
     </row>
-    <row r="13" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
-      <c r="R13" s="12"/>
-      <c r="S13" s="12"/>
-      <c r="T13" s="12"/>
-      <c r="U13" s="12"/>
-      <c r="V13" s="14">
+    <row r="13" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="24"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="10"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="12">
         <f>IF(B13="",0,VLOOKUP(T13,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W13"/>
     </row>
-    <row r="14" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="12"/>
-      <c r="R14" s="12"/>
-      <c r="S14" s="12"/>
-      <c r="T14" s="12"/>
-      <c r="U14" s="12"/>
-      <c r="V14" s="14">
+    <row r="14" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="24"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="12">
         <f>IF(B14="",0,VLOOKUP(T14,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W14"/>
     </row>
-    <row r="15" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="12"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="12"/>
-      <c r="Q15" s="12"/>
-      <c r="R15" s="12"/>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="12"/>
-      <c r="V15" s="14">
+    <row r="15" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="24"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="12">
         <f>IF(B15="",0,VLOOKUP(T15,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W15"/>
     </row>
-    <row r="16" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="12"/>
-      <c r="O16" s="12"/>
-      <c r="P16" s="12"/>
-      <c r="Q16" s="12"/>
-      <c r="R16" s="12"/>
-      <c r="S16" s="12"/>
-      <c r="T16" s="12"/>
-      <c r="U16" s="12"/>
-      <c r="V16" s="14">
+    <row r="16" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="12">
         <f>IF(B16="",0,VLOOKUP(T16,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W16"/>
     </row>
-    <row r="17" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="12"/>
-      <c r="Q17" s="12"/>
-      <c r="R17" s="12"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="12"/>
-      <c r="U17" s="12"/>
-      <c r="V17" s="14">
+    <row r="17" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="24"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="10"/>
+      <c r="V17" s="12">
         <f>IF(B17="",0,VLOOKUP(T17,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W17"/>
     </row>
-    <row r="18" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="12"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="12"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="14">
+    <row r="18" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="23"/>
+      <c r="P18" s="24"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="12">
         <f>IF(B18="",0,VLOOKUP(T18,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W18"/>
     </row>
-    <row r="19" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="12"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-      <c r="Q19" s="12"/>
-      <c r="R19" s="12"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="12"/>
-      <c r="U19" s="12"/>
-      <c r="V19" s="14">
+    <row r="19" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="24"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="12">
         <f>IF(B19="",0,VLOOKUP(T19,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="W19"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="17" type="noConversion"/>
+  <conditionalFormatting sqref="I1:I1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q19" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
       <formula1>"KG, L, Ds"</formula1>
@@ -1513,9 +1498,9 @@
         <v>30</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1523,7 +1508,7 @@
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="14" t="s">
         <v>25</v>
       </c>
       <c r="D2" s="6"/>
@@ -1532,56 +1517,56 @@
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="14" t="s">
         <v>25</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="16"/>
+        <v>35</v>
+      </c>
+      <c r="F3" s="14"/>
     </row>
     <row r="4" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>46</v>
+      <c r="B4" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>46</v>
+      <c r="B5" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>46</v>
+      <c r="B6" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>46</v>
+      <c r="B7" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F7"/>
     </row>
@@ -1589,11 +1574,11 @@
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="14" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F8"/>
     </row>
@@ -1601,7 +1586,7 @@
       <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="14" t="s">
         <v>27</v>
       </c>
       <c r="D9"/>
@@ -1611,7 +1596,7 @@
       <c r="A10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="14" t="s">
         <v>27</v>
       </c>
       <c r="D10"/>
@@ -1621,7 +1606,7 @@
       <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="14" t="s">
         <v>27</v>
       </c>
       <c r="D11"/>
@@ -1631,7 +1616,7 @@
       <c r="A12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14" t="s">
         <v>27</v>
       </c>
       <c r="D12"/>
@@ -1641,7 +1626,7 @@
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="14" t="s">
         <v>28</v>
       </c>
       <c r="D13"/>
@@ -1651,7 +1636,7 @@
       <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>28</v>
       </c>
       <c r="D14"/>

</xml_diff>

<commit_message>
Acrescido automação de RAs
</commit_message>
<xml_diff>
--- a/Plan_RNC.xlsx
+++ b/Plan_RNC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\AUTO-RNC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0915D352-746C-4E15-983D-67667789C21F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291D0F20-7480-4C2F-88E0-7FD3D61DF802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,41 +210,41 @@
     <t>RESUMO-RAPIDO</t>
   </si>
   <si>
-    <t>VZP NITRO</t>
-  </si>
-  <si>
     <t>NITRO</t>
   </si>
   <si>
-    <t>DATA DE FRABRICAÇÃO DIVERGENTE</t>
-  </si>
-  <si>
-    <t>00104</t>
-  </si>
-  <si>
-    <t>SPEED GRAMINEA SCX25KG</t>
-  </si>
-  <si>
-    <t>74771/26</t>
-  </si>
-  <si>
-    <t>a05</t>
-  </si>
-  <si>
     <t>Cuiabá</t>
   </si>
   <si>
-    <t>VZP TRANSF CBA</t>
-  </si>
-  <si>
-    <t>Durante o recebimento proveniente da unidade NITRO VZP, realizado pela transportadora MMCM, veículo placa SUF-2B15, foi identificada a seguinte não conformidade: A) O produto SPEED GRAMINEA SCX25KG (NF 10670, Lote 74771/26) apresentou divergência na informação de data de fabricação. No momento da conferência física, constatou-se que a data gravada nas sacarias é 04/03/2026, enquanto o documento fiscal (NF) indica a data de 06/03/2026. Esta inconsistência entre o físico e o faturado compromete a rastreabilidade e o padrão de conformidade Nitro.</t>
+    <t>Caixas amassadas</t>
+  </si>
+  <si>
+    <t>a01</t>
+  </si>
+  <si>
+    <t>03824</t>
+  </si>
+  <si>
+    <t>SPEED CX02X10KG</t>
+  </si>
+  <si>
+    <t>HORT TRANSF CBA</t>
+  </si>
+  <si>
+    <t>HORT</t>
+  </si>
+  <si>
+    <t>69177/25</t>
+  </si>
+  <si>
+    <t>Durante a descarga da transferência proveniente da unidade de Hortolândia para a unidade de Cuiabá, realizada pela transportadora Fantinato, veículo placa FTG0F13, foi identificada a seguinte não conformidade: A) O produto SPEED CX02X10KG (NF 10817, Lote 69177/25) apresentou caixas amassadas no momento da conferência. A avaria na embalagem secundária caracteriza o descumprimento do padrão Nitro de transporte e integridade da carga, sendo necessária a ressalva para registro de qualidade.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,10 +342,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FFFFFF00"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -354,22 +351,7 @@
       <b/>
       <u/>
       <sz val="12"/>
-      <color rgb="FFFFC000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
+      <color rgb="FFFFFF00"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -381,12 +363,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -409,6 +385,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -449,17 +431,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -485,7 +467,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -495,27 +477,9 @@
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -524,6 +488,18 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -819,12 +795,13 @@
   <dimension ref="A1:W19"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="22" width="25.77734375" style="1" customWidth="1"/>
+    <col min="1" max="21" width="25.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="25.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="23" max="23" width="0" hidden="1" customWidth="1"/>
     <col min="24" max="16384" width="8.88671875" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="16" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="22" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>48</v>
       </c>
@@ -834,13 +811,13 @@
       <c r="C1" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="20" t="s">
@@ -861,113 +838,113 @@
       <c r="L1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="21" t="s">
+      <c r="N1" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="19" t="s">
+      <c r="Q1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="19" t="s">
+      <c r="R1" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="S1" s="22" t="s">
+      <c r="S1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="19" t="s">
+      <c r="T1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="19" t="s">
+      <c r="U1" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="V1" s="19" t="s">
+      <c r="V1" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="W1" s="17"/>
+      <c r="W1" s="21"/>
     </row>
     <row r="2" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="18">
-        <v>355</v>
-      </c>
-      <c r="C2" s="18" t="s">
+      <c r="B2" s="16">
+        <v>356</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" s="10" t="s">
+      <c r="I2" s="10">
+        <v>10817</v>
+      </c>
+      <c r="J2" s="11">
+        <v>45842</v>
+      </c>
+      <c r="K2" s="11">
+        <v>46938</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="I2" s="10">
-        <v>10670</v>
-      </c>
-      <c r="J2" s="11">
-        <v>46087</v>
-      </c>
-      <c r="K2" s="11">
-        <v>46816</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="M2" s="11">
-        <v>46085</v>
+        <v>45842</v>
       </c>
       <c r="N2" s="11">
-        <v>46816</v>
-      </c>
-      <c r="O2" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="P2" s="24">
-        <v>30000</v>
+        <v>46938</v>
+      </c>
+      <c r="O2" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="P2" s="18">
+        <v>9800</v>
       </c>
       <c r="Q2" s="10" t="s">
         <v>33</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="S2" s="15" t="s">
         <v>58</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="V2" s="12" t="str">
         <f>IF(B2="",0,VLOOKUP(T2,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>PROCESSO</v>
+        <v xml:space="preserve">EMBALAGEM </v>
       </c>
       <c r="W2"/>
     </row>
     <row r="3" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="23"/>
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="17"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
       <c r="G3" s="10"/>
@@ -978,8 +955,8 @@
       <c r="L3" s="10"/>
       <c r="M3" s="11"/>
       <c r="N3" s="11"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="24"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="18"/>
       <c r="Q3" s="10"/>
       <c r="R3" s="10"/>
       <c r="S3" s="15"/>
@@ -992,10 +969,10 @@
       <c r="W3"/>
     </row>
     <row r="4" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="23"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
       <c r="G4" s="10"/>
@@ -1006,8 +983,8 @@
       <c r="L4" s="10"/>
       <c r="M4" s="11"/>
       <c r="N4" s="11"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="24"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="18"/>
       <c r="Q4" s="10"/>
       <c r="R4" s="10"/>
       <c r="S4" s="15"/>
@@ -1019,11 +996,11 @@
       </c>
       <c r="W4"/>
     </row>
-    <row r="5" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="23"/>
+    <row r="5" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="17"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="10"/>
@@ -1034,8 +1011,8 @@
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="24"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="18"/>
       <c r="Q5" s="10"/>
       <c r="R5" s="10"/>
       <c r="S5" s="15"/>
@@ -1048,10 +1025,10 @@
       <c r="W5"/>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="23"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
@@ -1062,8 +1039,8 @@
       <c r="L6" s="10"/>
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="24"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="18"/>
       <c r="Q6" s="10"/>
       <c r="R6" s="10"/>
       <c r="S6" s="15"/>
@@ -1076,10 +1053,10 @@
       <c r="W6"/>
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="23"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="17"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -1090,8 +1067,8 @@
       <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="18"/>
       <c r="Q7" s="10"/>
       <c r="R7" s="10"/>
       <c r="S7" s="10"/>
@@ -1104,10 +1081,10 @@
       <c r="W7"/>
     </row>
     <row r="8" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="23"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="17"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
@@ -1118,8 +1095,8 @@
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="24"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="18"/>
       <c r="Q8" s="10"/>
       <c r="R8" s="10"/>
       <c r="S8" s="10"/>
@@ -1132,10 +1109,10 @@
       <c r="W8"/>
     </row>
     <row r="9" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="23"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="17"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
@@ -1146,8 +1123,8 @@
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="24"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="18"/>
       <c r="Q9" s="10"/>
       <c r="R9" s="10"/>
       <c r="S9" s="10"/>
@@ -1160,10 +1137,10 @@
       <c r="W9"/>
     </row>
     <row r="10" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="23"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
@@ -1174,8 +1151,8 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="24"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="18"/>
       <c r="Q10" s="10"/>
       <c r="R10" s="10"/>
       <c r="S10" s="10"/>
@@ -1188,10 +1165,10 @@
       <c r="W10"/>
     </row>
     <row r="11" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="23"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
@@ -1202,8 +1179,8 @@
       <c r="L11" s="10"/>
       <c r="M11" s="10"/>
       <c r="N11" s="10"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="24"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="18"/>
       <c r="Q11" s="10"/>
       <c r="R11" s="10"/>
       <c r="S11" s="10"/>
@@ -1216,10 +1193,10 @@
       <c r="W11"/>
     </row>
     <row r="12" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="23"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
@@ -1230,8 +1207,8 @@
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="24"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="18"/>
       <c r="Q12" s="10"/>
       <c r="R12" s="10"/>
       <c r="S12" s="10"/>
@@ -1244,10 +1221,10 @@
       <c r="W12"/>
     </row>
     <row r="13" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="23"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -1258,8 +1235,8 @@
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
       <c r="N13" s="10"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="24"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="18"/>
       <c r="Q13" s="10"/>
       <c r="R13" s="10"/>
       <c r="S13" s="10"/>
@@ -1272,10 +1249,10 @@
       <c r="W13"/>
     </row>
     <row r="14" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="23"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -1286,8 +1263,8 @@
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="24"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="18"/>
       <c r="Q14" s="10"/>
       <c r="R14" s="10"/>
       <c r="S14" s="10"/>
@@ -1300,10 +1277,10 @@
       <c r="W14"/>
     </row>
     <row r="15" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="23"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -1314,8 +1291,8 @@
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="24"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="18"/>
       <c r="Q15" s="10"/>
       <c r="R15" s="10"/>
       <c r="S15" s="10"/>
@@ -1328,10 +1305,10 @@
       <c r="W15"/>
     </row>
     <row r="16" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="23"/>
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
@@ -1342,8 +1319,8 @@
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="24"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="18"/>
       <c r="Q16" s="10"/>
       <c r="R16" s="10"/>
       <c r="S16" s="10"/>
@@ -1356,10 +1333,10 @@
       <c r="W16"/>
     </row>
     <row r="17" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="18"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="23"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -1370,8 +1347,8 @@
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
       <c r="N17" s="10"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="24"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="18"/>
       <c r="Q17" s="10"/>
       <c r="R17" s="10"/>
       <c r="S17" s="10"/>
@@ -1384,10 +1361,10 @@
       <c r="W17"/>
     </row>
     <row r="18" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="18"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="23"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
@@ -1398,8 +1375,8 @@
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="10"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="24"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="18"/>
       <c r="Q18" s="10"/>
       <c r="R18" s="10"/>
       <c r="S18" s="10"/>
@@ -1412,10 +1389,10 @@
       <c r="W18"/>
     </row>
     <row r="19" spans="1:23" s="9" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="18"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="23"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="17"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -1426,8 +1403,8 @@
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
       <c r="N19" s="10"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="24"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="18"/>
       <c r="Q19" s="10"/>
       <c r="R19" s="10"/>
       <c r="S19" s="10"/>
@@ -1440,7 +1417,8 @@
       <c r="W19"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="I1:I1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Arquivos do desktop + Correção de bugs
</commit_message>
<xml_diff>
--- a/Plan_RNC.xlsx
+++ b/Plan_RNC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976FC62D-F473-42EC-ACD9-B3D280A007AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48DC7E4-1854-4E14-B3DD-8E43EB314D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="69">
   <si>
     <t>NUMERO-NF</t>
   </si>
@@ -222,52 +222,52 @@
     <t>NITRO</t>
   </si>
   <si>
-    <t>UM GALÃO DE 5L COM VAZAMENTO</t>
-  </si>
-  <si>
-    <t>CAIXAS AMASSADAS, RASGADAS E DOIS GALÕES DE 10L COM VAZAMENTO</t>
-  </si>
-  <si>
-    <t>CAIXAS AMASSADAS E UM GALÃO DE 5L COM VAZAMENTO</t>
-  </si>
-  <si>
-    <t>DATA DE VALIDADE DIVERTE DA NF</t>
-  </si>
-  <si>
-    <t>1000041</t>
-  </si>
-  <si>
-    <t>05043</t>
-  </si>
-  <si>
-    <t>510052</t>
-  </si>
-  <si>
-    <t>ELMO CX02X05L</t>
-  </si>
-  <si>
-    <t>DUNNA CX02X05L</t>
-  </si>
-  <si>
-    <t>ARRANK CX02X05L</t>
-  </si>
-  <si>
-    <t>FB1324</t>
-  </si>
-  <si>
-    <t>FB1125</t>
-  </si>
-  <si>
-    <t>SKB0324.B</t>
-  </si>
-  <si>
-    <t>74604/26</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>X</t>
+    <t>DATA E LOTE DIVERGENTE</t>
+  </si>
+  <si>
+    <t>2 SACARIAS AVARIADAS</t>
+  </si>
+  <si>
+    <t>04945</t>
+  </si>
+  <si>
+    <t>05340</t>
+  </si>
+  <si>
+    <t>510009</t>
+  </si>
+  <si>
+    <t>SPEED SCX25KG</t>
+  </si>
+  <si>
+    <t>LOADER SCX20KG</t>
+  </si>
+  <si>
+    <t>BOROMAG CX02X10KG</t>
+  </si>
+  <si>
+    <t>Lote WMS</t>
+  </si>
+  <si>
+    <t>75646/26</t>
+  </si>
+  <si>
+    <t>74797/26</t>
+  </si>
+  <si>
+    <t>75574/26</t>
+  </si>
+  <si>
+    <t>75720/26</t>
+  </si>
+  <si>
+    <t>70809/25</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -934,19 +934,19 @@
         <v>53</v>
       </c>
       <c r="B2" s="17">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>48</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E2" s="17" t="s">
         <v>49</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G2" s="17" t="s">
         <v>50</v>
@@ -955,68 +955,68 @@
         <v>51</v>
       </c>
       <c r="I2" s="17">
-        <v>10778</v>
+        <v>10810</v>
       </c>
       <c r="J2" s="18">
-        <v>45551</v>
+        <v>45482</v>
       </c>
       <c r="K2" s="18">
-        <v>46108</v>
+        <v>46212</v>
       </c>
       <c r="L2" s="16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M2" s="18">
-        <v>45551</v>
+        <v>46100</v>
       </c>
       <c r="N2" s="18">
-        <v>46108</v>
+        <v>47196</v>
       </c>
       <c r="O2" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P2" s="19">
-        <v>5</v>
+        <v>5000</v>
       </c>
       <c r="Q2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="R2" s="17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S2" s="20" t="s">
         <v>68</v>
       </c>
       <c r="T2" s="17" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="U2" s="17" t="s">
         <v>52</v>
       </c>
       <c r="V2" s="10" t="str">
         <f>IF(B2="",0,VLOOKUP(T2,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>AVARIA</v>
+        <v>PROCESSO</v>
       </c>
       <c r="W2"/>
     </row>
     <row r="3" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="17">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>48</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E3" s="17" t="s">
         <v>49</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G3" s="17" t="s">
         <v>50</v>
@@ -1025,68 +1025,68 @@
         <v>51</v>
       </c>
       <c r="I3" s="17">
-        <v>10778</v>
+        <v>10810</v>
       </c>
       <c r="J3" s="18">
-        <v>45900</v>
+        <v>45482</v>
       </c>
       <c r="K3" s="18">
-        <v>46446</v>
+        <v>46212</v>
       </c>
       <c r="L3" s="16" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="M3" s="18">
-        <v>45900</v>
+        <v>46094</v>
       </c>
       <c r="N3" s="18">
-        <v>46446</v>
+        <v>47190</v>
       </c>
       <c r="O3" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P3" s="19">
-        <v>160</v>
+        <v>2500</v>
       </c>
       <c r="Q3" s="17" t="s">
         <v>67</v>
       </c>
       <c r="R3" s="17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S3" s="20" t="s">
         <v>68</v>
       </c>
       <c r="T3" s="17" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="U3" s="17" t="s">
         <v>52</v>
       </c>
       <c r="V3" s="10" t="str">
         <f>IF(B3="",0,VLOOKUP(T3,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>AVARIA</v>
+        <v>PROCESSO</v>
       </c>
       <c r="W3"/>
     </row>
     <row r="4" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B4" s="17">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>49</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G4" s="17" t="s">
         <v>50</v>
@@ -1095,68 +1095,68 @@
         <v>51</v>
       </c>
       <c r="I4" s="17">
-        <v>10778</v>
+        <v>10810</v>
       </c>
       <c r="J4" s="18">
-        <v>45505</v>
+        <v>45482</v>
       </c>
       <c r="K4" s="18">
-        <v>46108</v>
+        <v>46212</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="M4" s="18">
-        <v>45505</v>
+        <v>46101</v>
       </c>
       <c r="N4" s="18">
-        <v>46108</v>
+        <v>47197</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P4" s="19">
-        <v>115</v>
+        <v>2500</v>
       </c>
       <c r="Q4" s="17" t="s">
         <v>67</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S4" s="20" t="s">
         <v>68</v>
       </c>
       <c r="T4" s="17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U4" s="17" t="s">
         <v>52</v>
       </c>
       <c r="V4" s="10" t="str">
         <f>IF(B4="",0,VLOOKUP(T4,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v xml:space="preserve">EMBALAGEM </v>
+        <v>PROCESSO</v>
       </c>
       <c r="W4"/>
     </row>
     <row r="5" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B5" s="17">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>48</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>49</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G5" s="17" t="s">
         <v>50</v>
@@ -1165,75 +1165,117 @@
         <v>51</v>
       </c>
       <c r="I5" s="17">
-        <v>10778</v>
+        <v>10810</v>
       </c>
       <c r="J5" s="18">
-        <v>46090</v>
+        <v>45985</v>
       </c>
       <c r="K5" s="18">
-        <v>46821</v>
+        <v>2958465</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="M5" s="18">
-        <v>46090</v>
+        <v>46106</v>
       </c>
       <c r="N5" s="18">
-        <v>47186</v>
+        <v>47202</v>
       </c>
       <c r="O5" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P5" s="19">
-        <v>10800</v>
+        <v>9000</v>
       </c>
       <c r="Q5" s="17" t="s">
         <v>67</v>
       </c>
       <c r="R5" s="17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S5" s="20" t="s">
         <v>68</v>
       </c>
       <c r="T5" s="17" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="U5" s="17" t="s">
         <v>52</v>
       </c>
       <c r="V5" s="10" t="str">
         <f>IF(B5="",0,VLOOKUP(T5,Planilha1!$A$2:$B$14,2,FALSE))</f>
+        <v>AVARIA</v>
+      </c>
+      <c r="W5"/>
+    </row>
+    <row r="6" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="23">
+        <v>367</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" s="23">
+        <v>10810</v>
+      </c>
+      <c r="J6" s="25">
+        <v>45756</v>
+      </c>
+      <c r="K6" s="25">
+        <v>2958465</v>
+      </c>
+      <c r="L6" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="M6" s="25">
+        <v>45901</v>
+      </c>
+      <c r="N6" s="25">
+        <v>46997</v>
+      </c>
+      <c r="O6" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="26">
+        <v>4900</v>
+      </c>
+      <c r="Q6" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="R6" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="S6" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="T6" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="U6" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="V6" s="28" t="str">
+        <f>IF(B6="",0,VLOOKUP(T6,Planilha1!$A$2:$B$14,2,FALSE))</f>
         <v>PROCESSO</v>
-      </c>
-      <c r="W5"/>
-    </row>
-    <row r="6" spans="1:23" s="9" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="24"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="23"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="27"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="V6" s="28">
-        <f>IF(B6="",0,VLOOKUP(T6,Planilha1!$A$2:$B$14,2,FALSE))</f>
-        <v>0</v>
       </c>
       <c r="W6"/>
     </row>

</xml_diff>